<commit_message>
Config erweitert, Versionen angehoben, VESPA-Url Arg aktualisiert
</commit_message>
<xml_diff>
--- a/KVR_Parkausweise_Performer/Data/Config.xlsx
+++ b/KVR_Parkausweise_Performer/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ex.dwight\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_PAU\KVR_Parkausweise_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6543B54-2CB7-4EFC-9B7F-BCBFBD3C66A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3568E4BB-8D1F-4D33-A7CD-B22AB7E61883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4245" yWindow="4245" windowWidth="45705" windowHeight="15285" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22155" yWindow="3675" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="83">
   <si>
     <t>Name</t>
   </si>
@@ -234,33 +234,12 @@
     <t>CreateQueueReport</t>
   </si>
   <si>
-    <t>SharedMailbox</t>
-  </si>
-  <si>
-    <t>MailfolderSuccess</t>
-  </si>
-  <si>
-    <t>MailfolderFailed</t>
-  </si>
-  <si>
-    <t>MailfolderInbox</t>
-  </si>
-  <si>
     <t>rpa010_Robot Account</t>
   </si>
   <si>
-    <t>URL_Vespa</t>
-  </si>
-  <si>
-    <t>pathdownload</t>
-  </si>
-  <si>
     <t>msedge,excel</t>
   </si>
   <si>
-    <t>MailfolderPostversand</t>
-  </si>
-  <si>
     <t>rpa010_ParkausweiseQueue</t>
   </si>
   <si>
@@ -289,6 +268,12 @@
   </si>
   <si>
     <t>rpa010_ReplaceTitel</t>
+  </si>
+  <si>
+    <t>rpa010_WebexRoomID</t>
+  </si>
+  <si>
+    <t>rpa010_WebexApiUrl</t>
   </si>
 </sst>
 </file>
@@ -665,12 +650,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -712,13 +697,13 @@
         <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -728,7 +713,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="28.8">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1742,12 +1727,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1784,7 +1769,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1795,7 +1780,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="30">
+    <row r="3" spans="1:26" ht="28.8">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1806,7 +1791,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="45">
+    <row r="4" spans="1:26" ht="43.2">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1817,19 +1802,19 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" ht="14.4">
       <c r="A5" t="s">
         <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" ht="14.4">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -1856,7 +1841,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" ht="14.4">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -1867,13 +1852,13 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:26"/>
-    <row r="12" spans="1:26">
+    <row r="11" spans="1:26" ht="14.4"/>
+    <row r="12" spans="1:26" ht="14.4">
       <c r="A12" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" ht="14.4">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -1884,7 +1869,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" ht="14.4">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -1895,7 +1880,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" ht="14.4">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -1906,7 +1891,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:26" ht="14.4">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -1917,7 +1902,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" ht="14.4">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -2019,7 +2004,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:3" ht="45">
+    <row r="29" spans="1:3" ht="28.8">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -2033,18 +2018,18 @@
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1"/>
@@ -3023,12 +3008,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z999"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="60.33203125" customWidth="1"/>
+    <col min="4" max="26" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3069,70 +3054,84 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" t="s">
+        <v>82</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>